<commit_message>
Recale la feuille sur les règles du SDK et réexporte le jeu Stake
- 1 trophée max par rouleau dans la feuille (formules + simulateur), comme sur les bandes du SDK
- Trophée base 110, bonus buy 69x : RTP simulé 95,7 % ± 1,9 %, bonus 1/148
- Export SDK régénéré ; gains feuille = SDK sur 20 000 grilles pour les 4 modes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014K11WNgkEUnnGsVcri14bC
</commit_message>
<xml_diff>
--- a/wild_side_school/wild_side_school_math.xlsx
+++ b/wild_side_school/wild_side_school_math.xlsx
@@ -91,7 +91,7 @@
     <t xml:space="preserve">• Les trophées et les autres globes ne sont pas remplacés par les multis. Une ligne ou une way 100 % wild paie comme le 1er symbole PAY de la paytable (le Singe).</t>
   </si>
   <si>
-    <t xml:space="preserve">• Les cases sont tirées indépendamment selon les poids de chaque rouleau (modèle à poids, pas de bandes de rouleaux). Les multis ne restent pas collés d'un FS à l'autre.</t>
+    <t xml:space="preserve">• Chaque case suit les poids de son rouleau, avec au plus 1 trophée par rouleau (comme sur les bandes du math SDK de Stake Engine, voir le dossier stake_math). Les multis ne restent pas collés d'un FS à l'autre.</t>
   </si>
   <si>
     <t xml:space="preserve">• Les valeurs de la paytable, des poids et des multis sont des valeurs de départ calées pour ~96 % de RTP. Ce ne sont PAS les valeurs officielles du jeu (non publiées).</t>
@@ -541,7 +541,7 @@
     <t xml:space="preserve">RTP des gains — calcul analytique exact HORS globe/multis</t>
   </si>
   <si>
-    <t xml:space="preserve">WAYS : E[ways de longueur k] = Π(lignes × p_r, r ≤ k) × (1 − p_{k+1})^lignes. LINES : nb lignes × Π(p_r, r ≤ k) × (1 − p_{k+1}). Le globe et ses multis sont ajoutés par le simulateur.</t>
+    <t xml:space="preserve">WAYS : E[ways de longueur k] = Π(lignes × p_r, r ≤ k) × P(aucun sur le rouleau k+1). LINES : nb lignes × Π(p_r, r ≤ k) × (1 − p_{k+1}). Le globe et ses multis sont ajoutés par le simulateur.</t>
   </si>
   <si>
     <t xml:space="preserve">JEU DE BASE — RTP par spin hors globe</t>
@@ -586,7 +586,7 @@
     <t xml:space="preserve">Fréquence du bonus, nombre de FS, fréquence du globe</t>
   </si>
   <si>
-    <t xml:space="preserve">Nombre de trophées sur la grille = somme de 5 lois binomiales (une par rouleau), calculée par convolution.</t>
+    <t xml:space="preserve">Au plus 1 trophée par rouleau (probabilité = lignes × p). Total sur la grille calculé par convolution des 5 rouleaux.</t>
   </si>
   <si>
     <t xml:space="preserve">Probabilité d'une case</t>
@@ -607,7 +607,7 @@
     <t xml:space="preserve">Globe — FS</t>
   </si>
   <si>
-    <t xml:space="preserve">Loi du nombre de trophées par rouleau (jeu de base)</t>
+    <t xml:space="preserve">Nombre de trophées par rouleau, jeu de base (au plus 1 par rouleau, comme sur les bandes du SDK)</t>
   </si>
   <si>
     <t xml:space="preserve">k</t>
@@ -682,7 +682,7 @@
     <t xml:space="preserve">Date de la simulation</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-09 18:25</t>
+    <t xml:space="preserve">2026-10-09 19:03</t>
   </si>
   <si>
     <t xml:space="preserve">0 x</t>
@@ -1439,7 +1439,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>210</v>
       </c>
       <c r="G5" s="47" t="n">
-        <v>0.597609</v>
+        <v>0.599854</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1576,7 +1576,7 @@
         <v>211</v>
       </c>
       <c r="G6" s="47" t="n">
-        <v>0.3166115</v>
+        <v>0.315148</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1590,7 +1590,7 @@
         <v>213</v>
       </c>
       <c r="G7" s="47" t="n">
-        <v>0.0769695</v>
+        <v>0.075864</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1598,13 +1598,13 @@
         <v>214</v>
       </c>
       <c r="B8" s="30" t="n">
-        <v>0.52667235</v>
+        <v>0.50225255</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>215</v>
       </c>
       <c r="G8" s="47" t="n">
-        <v>0.003793</v>
+        <v>0.004043</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1612,13 +1612,13 @@
         <v>51</v>
       </c>
       <c r="B9" s="30" t="n">
-        <v>0.424045725</v>
+        <v>0.4545129</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>216</v>
       </c>
       <c r="G9" s="47" t="n">
-        <v>0.0026655</v>
+        <v>0.002751</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1626,13 +1626,13 @@
         <v>52</v>
       </c>
       <c r="B10" s="30" t="n">
-        <v>0.950718075</v>
+        <v>0.95676545</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>217</v>
       </c>
       <c r="G10" s="47" t="n">
-        <v>0.002339</v>
+        <v>0.002329</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1640,13 +1640,13 @@
         <v>218</v>
       </c>
       <c r="B11" s="47" t="n">
-        <v>0.0186439732835432</v>
+        <v>0.0187553584492112</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>219</v>
       </c>
       <c r="G11" s="47" t="n">
-        <v>1.25E-005</v>
+        <v>1.1E-005</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1654,7 +1654,7 @@
         <v>57</v>
       </c>
       <c r="B12" s="30" t="n">
-        <v>0.402391</v>
+        <v>0.400146</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>220</v>
@@ -1668,7 +1668,7 @@
         <v>221</v>
       </c>
       <c r="B13" s="48" t="n">
-        <v>13.4523264663819</v>
+        <v>13.5326950438997</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="47"/>
@@ -1678,7 +1678,7 @@
         <v>38</v>
       </c>
       <c r="B14" s="22" t="n">
-        <v>161.394448030988</v>
+        <v>147.907114332199</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="47"/>
@@ -1688,7 +1688,7 @@
         <v>40</v>
       </c>
       <c r="B15" s="48" t="n">
-        <v>24.5331665590704</v>
+        <v>24.351723117882</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1696,7 +1696,7 @@
         <v>60</v>
       </c>
       <c r="B16" s="26" t="n">
-        <v>68.438625726275</v>
+        <v>67.2256914657595</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1704,7 +1704,7 @@
         <v>61</v>
       </c>
       <c r="B17" s="26" t="n">
-        <v>69.285536</v>
+        <v>66.7649335</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1712,7 +1712,7 @@
         <v>222</v>
       </c>
       <c r="B18" s="30" t="n">
-        <v>0.962299111111111</v>
+        <v>0.967607731884058</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1720,7 +1720,7 @@
         <v>223</v>
       </c>
       <c r="B19" s="26" t="n">
-        <v>4475.7</v>
+        <v>2963.9</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1736,7 +1736,7 @@
         <v>44</v>
       </c>
       <c r="B21" s="30" t="n">
-        <v>0.004152</v>
+        <v>0.0041265</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1744,7 +1744,7 @@
         <v>225</v>
       </c>
       <c r="B22" s="30" t="n">
-        <v>0.2591201</v>
+        <v>0.2380552</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1774,10 +1774,10 @@
         <v>112</v>
       </c>
       <c r="C27" s="30" t="n">
-        <v>0.092497</v>
+        <v>0.0846065</v>
       </c>
       <c r="D27" s="30" t="n">
-        <v>0.139397</v>
+        <v>0.149525</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1788,10 +1788,10 @@
         <v>115</v>
       </c>
       <c r="C28" s="30" t="n">
-        <v>0.05200775</v>
+        <v>0.050493</v>
       </c>
       <c r="D28" s="30" t="n">
-        <v>0.06428875</v>
+        <v>0.0708165</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1802,10 +1802,10 @@
         <v>117</v>
       </c>
       <c r="C29" s="30" t="n">
-        <v>0.0607289500000015</v>
+        <v>0.0558431000000014</v>
       </c>
       <c r="D29" s="30" t="n">
-        <v>0.0596361</v>
+        <v>0.06374165</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1816,10 +1816,10 @@
         <v>119</v>
       </c>
       <c r="C30" s="30" t="n">
-        <v>0.0639165000000017</v>
+        <v>0.0601173000000013</v>
       </c>
       <c r="D30" s="30" t="n">
-        <v>0.0455474</v>
+        <v>0.0479198</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1830,10 +1830,10 @@
         <v>121</v>
       </c>
       <c r="C31" s="30" t="n">
-        <v>0.08221105000001</v>
+        <v>0.07976940000001</v>
       </c>
       <c r="D31" s="30" t="n">
-        <v>0.04133085</v>
+        <v>0.0427529</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1844,10 +1844,10 @@
         <v>123</v>
       </c>
       <c r="C32" s="30" t="n">
-        <v>0.0868599999999976</v>
+        <v>0.0847240499999971</v>
       </c>
       <c r="D32" s="30" t="n">
-        <v>0.039511125</v>
+        <v>0.04233255</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1858,10 +1858,10 @@
         <v>125</v>
       </c>
       <c r="C33" s="30" t="n">
-        <v>0.0884510999999943</v>
+        <v>0.086699199999993</v>
       </c>
       <c r="D33" s="30" t="n">
-        <v>0.0343345</v>
+        <v>0.0374245</v>
       </c>
     </row>
   </sheetData>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="B12" s="13" t="n">
         <f aca="false">Calc_Gains!K12</f>
-        <v>0.2685949212761</v>
+        <v>0.265529063584556</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>36</v>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="B14" s="10" t="n">
         <f aca="false">Calc_Bonus!I22</f>
-        <v>160.967018789321</v>
+        <v>147.377657908019</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>39</v>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B15" s="15" t="n">
         <f aca="false">Calc_Bonus!I29</f>
-        <v>24.5556276828887</v>
+        <v>24.3627818075392</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>39</v>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="B17" s="16" t="n">
         <f aca="false">IF(ISNUMBER(Calc_Bonus!I29),Calc_Bonus!I21*Calc_Bonus!I29*Calc_Gains!K24,"-")</f>
-        <v>0.0381538501092052</v>
+        <v>0.0413446628894224</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>43</v>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">Calc_Bonus!I32</f>
-        <v>0.00419491142248873</v>
+        <v>0.00418087742329565</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>39</v>
@@ -2093,7 +2093,7 @@
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">Simulation!B8</f>
-        <v>0.52667235</v>
+        <v>0.50225255</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>50</v>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="B24" s="7" t="n">
         <f aca="false">Simulation!B9</f>
-        <v>0.424045725</v>
+        <v>0.4545129</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>50</v>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="B25" s="13" t="n">
         <f aca="false">Simulation!B10</f>
-        <v>0.950718075</v>
+        <v>0.95676545</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>50</v>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="B26" s="17" t="n">
         <f aca="false">IF(ISNUMBER(Simulation!B10),Simulation!B10-RTP_CIBLE,"-")</f>
-        <v>-0.00928192499999991</v>
+        <v>-0.00323455000000006</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>54</v>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="B28" s="7" t="n">
         <f aca="false">Simulation!B12</f>
-        <v>0.402391</v>
+        <v>0.400146</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>50</v>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="B29" s="15" t="n">
         <f aca="false">Simulation!B13</f>
-        <v>13.4523264663819</v>
+        <v>13.5326950438997</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>50</v>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="B30" s="10" t="n">
         <f aca="false">Simulation!B14</f>
-        <v>161.394448030988</v>
+        <v>147.907114332199</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>50</v>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="B31" s="19" t="n">
         <f aca="false">Simulation!B16</f>
-        <v>68.438625726275</v>
+        <v>67.2256914657595</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>50</v>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="B32" s="19" t="n">
         <f aca="false">Simulation!B17</f>
-        <v>69.285536</v>
+        <v>66.7649335</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>50</v>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="B33" s="7" t="n">
         <f aca="false">Simulation!B18</f>
-        <v>0.962299111111111</v>
+        <v>0.967607731884058</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>50</v>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="B34" s="20" t="n">
         <f aca="false">IF(ISNUMBER(Simulation!B17),Simulation!B17/RTP_CIBLE,"-")</f>
-        <v>72.1724333333333</v>
+        <v>69.5468057291667</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>64</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="B35" s="19" t="n">
         <f aca="false">Simulation!B19</f>
-        <v>4475.7</v>
+        <v>2963.9</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>50</v>
@@ -2416,7 +2416,7 @@
         <v>90</v>
       </c>
       <c r="B16" s="21" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>91</v>
@@ -3845,23 +3845,23 @@
       </c>
       <c r="I5" s="30" t="n">
         <f aca="false">IF(C$14=0,0,C5/C$14)</f>
-        <v>0.0513610683102209</v>
+        <v>0.0511858044702269</v>
       </c>
       <c r="J5" s="30" t="n">
         <f aca="false">IF(D$14=0,0,D5/D$14)</f>
-        <v>0.054505195026401</v>
+        <v>0.0543201493804108</v>
       </c>
       <c r="K5" s="30" t="n">
         <f aca="false">IF(E$14=0,0,E5/E$14)</f>
-        <v>0.0573259146855505</v>
+        <v>0.0571332549151403</v>
       </c>
       <c r="L5" s="30" t="n">
         <f aca="false">IF(F$14=0,0,F5/F$14)</f>
-        <v>0.059890201297621</v>
+        <v>0.0596915934339247</v>
       </c>
       <c r="M5" s="30" t="n">
         <f aca="false">IF(G$14=0,0,G5/G$14)</f>
-        <v>0.0623871285503201</v>
+        <v>0.0621829487808869</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3890,23 +3890,23 @@
       </c>
       <c r="I6" s="30" t="n">
         <f aca="false">IF(C$14=0,0,C6/C$14)</f>
-        <v>0.0770416024653313</v>
+        <v>0.0767787067053404</v>
       </c>
       <c r="J6" s="30" t="n">
         <f aca="false">IF(D$14=0,0,D6/D$14)</f>
-        <v>0.0783512178504514</v>
+        <v>0.0780852147343405</v>
       </c>
       <c r="K6" s="30" t="n">
         <f aca="false">IF(E$14=0,0,E6/E$14)</f>
-        <v>0.0809307030854831</v>
+        <v>0.0806587128213746</v>
       </c>
       <c r="L6" s="30" t="n">
         <f aca="false">IF(F$14=0,0,F6/F$14)</f>
-        <v>0.0831808351355848</v>
+        <v>0.082904990880451</v>
       </c>
       <c r="M6" s="30" t="n">
         <f aca="false">IF(G$14=0,0,G6/G$14)</f>
-        <v>0.0853718601214907</v>
+        <v>0.0850924562264769</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3935,23 +3935,23 @@
       </c>
       <c r="I7" s="30" t="n">
         <f aca="false">IF(C$14=0,0,C7/C$14)</f>
-        <v>0.102722136620442</v>
+        <v>0.102371608940454</v>
       </c>
       <c r="J7" s="30" t="n">
         <f aca="false">IF(D$14=0,0,D7/D$14)</f>
-        <v>0.102197240674502</v>
+        <v>0.10185028008827</v>
       </c>
       <c r="K7" s="30" t="n">
         <f aca="false">IF(E$14=0,0,E7/E$14)</f>
-        <v>0.104535491485416</v>
+        <v>0.104184170727609</v>
       </c>
       <c r="L7" s="30" t="n">
         <f aca="false">IF(F$14=0,0,F7/F$14)</f>
-        <v>0.106471468973548</v>
+        <v>0.106118388326977</v>
       </c>
       <c r="M7" s="30" t="n">
         <f aca="false">IF(G$14=0,0,G7/G$14)</f>
-        <v>0.108356591692661</v>
+        <v>0.108001963672067</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3980,23 +3980,23 @@
       </c>
       <c r="I8" s="30" t="n">
         <f aca="false">IF(C$14=0,0,C8/C$14)</f>
-        <v>0.136962848827256</v>
+        <v>0.136495478587272</v>
       </c>
       <c r="J8" s="30" t="n">
         <f aca="false">IF(D$14=0,0,D8/D$14)</f>
-        <v>0.136262987566002</v>
+        <v>0.135800373451027</v>
       </c>
       <c r="K8" s="30" t="n">
         <f aca="false">IF(E$14=0,0,E8/E$14)</f>
-        <v>0.134884505142472</v>
+        <v>0.134431188035624</v>
       </c>
       <c r="L8" s="30" t="n">
         <f aca="false">IF(F$14=0,0,F8/F$14)</f>
-        <v>0.136416569622359</v>
+        <v>0.13596418504394</v>
       </c>
       <c r="M8" s="30" t="n">
         <f aca="false">IF(G$14=0,0,G8/G$14)</f>
-        <v>0.137908389427023</v>
+        <v>0.13745704467354</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4025,23 +4025,23 @@
       </c>
       <c r="I9" s="30" t="n">
         <f aca="false">IF(C$14=0,0,C9/C$14)</f>
-        <v>0.188323917137476</v>
+        <v>0.187681283057499</v>
       </c>
       <c r="J9" s="30" t="n">
         <f aca="false">IF(D$14=0,0,D9/D$14)</f>
-        <v>0.187361607903253</v>
+        <v>0.186725513495162</v>
       </c>
       <c r="K9" s="30" t="n">
         <f aca="false">IF(E$14=0,0,E9/E$14)</f>
-        <v>0.185466194570899</v>
+        <v>0.184842883548983</v>
       </c>
       <c r="L9" s="30" t="n">
         <f aca="false">IF(F$14=0,0,F9/F$14)</f>
-        <v>0.182997837298286</v>
+        <v>0.182390979936992</v>
       </c>
       <c r="M9" s="30" t="n">
         <f aca="false">IF(G$14=0,0,G9/G$14)</f>
-        <v>0.180594319487769</v>
+        <v>0.180003272786778</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4070,23 +4070,23 @@
       </c>
       <c r="I10" s="30" t="n">
         <f aca="false">IF(C$14=0,0,C10/C$14)</f>
-        <v>0.205444273240883</v>
+        <v>0.204743217880908</v>
       </c>
       <c r="J10" s="30" t="n">
         <f aca="false">IF(D$14=0,0,D10/D$14)</f>
-        <v>0.204394481349004</v>
+        <v>0.20370056017654</v>
       </c>
       <c r="K10" s="30" t="n">
         <f aca="false">IF(E$14=0,0,E10/E$14)</f>
-        <v>0.202326757713708</v>
+        <v>0.201646782053436</v>
       </c>
       <c r="L10" s="30" t="n">
         <f aca="false">IF(F$14=0,0,F10/F$14)</f>
-        <v>0.199634004325403</v>
+        <v>0.198971978113082</v>
       </c>
       <c r="M10" s="30" t="n">
         <f aca="false">IF(G$14=0,0,G10/G$14)</f>
-        <v>0.197011984895748</v>
+        <v>0.196367206676485</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4115,23 +4115,23 @@
       </c>
       <c r="I11" s="30" t="n">
         <f aca="false">IF(C$14=0,0,C11/C$14)</f>
-        <v>0.22256462934429</v>
+        <v>0.221805152704317</v>
       </c>
       <c r="J11" s="30" t="n">
         <f aca="false">IF(D$14=0,0,D11/D$14)</f>
-        <v>0.221427354794754</v>
+        <v>0.220675606857919</v>
       </c>
       <c r="K11" s="30" t="n">
         <f aca="false">IF(E$14=0,0,E11/E$14)</f>
-        <v>0.219187320856517</v>
+        <v>0.218450680557889</v>
       </c>
       <c r="L11" s="30" t="n">
         <f aca="false">IF(F$14=0,0,F11/F$14)</f>
-        <v>0.21627017135252</v>
+        <v>0.215552976289173</v>
       </c>
       <c r="M11" s="30" t="n">
         <f aca="false">IF(G$14=0,0,G11/G$14)</f>
-        <v>0.213429650303727</v>
+        <v>0.212731140566192</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4144,39 +4144,39 @@
         <v>Trophée (bonus)</v>
       </c>
       <c r="C12" s="21" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="D12" s="21" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="F12" s="21" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="G12" s="21" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="I12" s="30" t="n">
         <f aca="false">IF(C$14=0,0,C12/C$14)</f>
-        <v>0.0154083204930663</v>
+        <v>0.0187681283057499</v>
       </c>
       <c r="J12" s="30" t="n">
         <f aca="false">IF(D$14=0,0,D12/D$14)</f>
-        <v>0.0153295861011753</v>
+        <v>0.0186725513495162</v>
       </c>
       <c r="K12" s="30" t="n">
         <f aca="false">IF(E$14=0,0,E12/E$14)</f>
-        <v>0.0151745068285281</v>
+        <v>0.0184842883548983</v>
       </c>
       <c r="L12" s="30" t="n">
         <f aca="false">IF(F$14=0,0,F12/F$14)</f>
-        <v>0.0149725503244053</v>
+        <v>0.0182390979936992</v>
       </c>
       <c r="M12" s="30" t="n">
         <f aca="false">IF(G$14=0,0,G12/G$14)</f>
-        <v>0.0147758988671811</v>
+        <v>0.0180003272786778</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4205,23 +4205,23 @@
       </c>
       <c r="I13" s="30" t="n">
         <f aca="false">IF(C$14=0,0,C13/C$14)</f>
-        <v>0.00017120356103407</v>
+        <v>0.00017061934823409</v>
       </c>
       <c r="J13" s="30" t="n">
         <f aca="false">IF(D$14=0,0,D13/D$14)</f>
-        <v>0.000170328734457503</v>
+        <v>0.000169750466813784</v>
       </c>
       <c r="K13" s="30" t="n">
         <f aca="false">IF(E$14=0,0,E13/E$14)</f>
-        <v>0.00016860563142809</v>
+        <v>0.00016803898504453</v>
       </c>
       <c r="L13" s="30" t="n">
         <f aca="false">IF(F$14=0,0,F13/F$14)</f>
-        <v>0.00016636167027117</v>
+        <v>0.000165809981760902</v>
       </c>
       <c r="M13" s="30" t="n">
         <f aca="false">IF(G$14=0,0,G13/G$14)</f>
-        <v>0.00016417665407979</v>
+        <v>0.000163639338897071</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4230,23 +4230,23 @@
       </c>
       <c r="C14" s="32" t="n">
         <f aca="false">SUM(C5:C13)</f>
-        <v>5841</v>
+        <v>5861</v>
       </c>
       <c r="D14" s="32" t="n">
         <f aca="false">SUM(D5:D13)</f>
-        <v>5871</v>
+        <v>5891</v>
       </c>
       <c r="E14" s="32" t="n">
         <f aca="false">SUM(E5:E13)</f>
-        <v>5931</v>
+        <v>5951</v>
       </c>
       <c r="F14" s="32" t="n">
         <f aca="false">SUM(F5:F13)</f>
-        <v>6011</v>
+        <v>6031</v>
       </c>
       <c r="G14" s="32" t="n">
         <f aca="false">SUM(G5:G13)</f>
-        <v>6091</v>
+        <v>6111</v>
       </c>
       <c r="I14" s="33" t="n">
         <f aca="false">SUM(I5:I13)</f>
@@ -5135,43 +5135,43 @@
       </c>
       <c r="C5" s="36" t="n">
         <f aca="false">Poids!I5</f>
-        <v>0.0513610683102209</v>
+        <v>0.0511858044702269</v>
       </c>
       <c r="D5" s="36" t="n">
         <f aca="false">Poids!J5</f>
-        <v>0.054505195026401</v>
+        <v>0.0543201493804108</v>
       </c>
       <c r="E5" s="36" t="n">
         <f aca="false">Poids!K5</f>
-        <v>0.0573259146855505</v>
+        <v>0.0571332549151403</v>
       </c>
       <c r="F5" s="36" t="n">
         <f aca="false">Poids!L5</f>
-        <v>0.059890201297621</v>
+        <v>0.0596915934339247</v>
       </c>
       <c r="G5" s="36" t="n">
         <f aca="false">Poids!M5</f>
-        <v>0.0623871285503201</v>
+        <v>0.0621829487808869</v>
       </c>
       <c r="H5" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C5*D5*E5*(1-F5)^NB_LIGNES,NB_PAYLINES*C5*D5*E5*(1-F5))</f>
-        <v>0.00301739047052251</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C5*D5*E5*((1-NB_LIGNES*Poids!$L$12)*(1-F5/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F5/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C5*D5*E5*(1-F5))</f>
+        <v>0.00298744397969826</v>
       </c>
       <c r="I5" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C5*D5*E5*F5*(1-G5)^NB_LIGNES,NB_PAYLINES*C5*D5*E5*F5*(1-G5))</f>
-        <v>0.000180232152115828</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C5*D5*E5*F5*((1-NB_LIGNES*Poids!$M$12)*(1-G5/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G5/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C5*D5*E5*F5*(1-G5))</f>
+        <v>0.000177852817023497</v>
       </c>
       <c r="J5" s="37" t="n">
         <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C5*D5*E5*F5*G5</f>
-        <v>1.19923337075844E-005</v>
+        <v>1.17927186300696E-005</v>
       </c>
       <c r="K5" s="30" t="n">
         <f aca="false">Paytable!D4*H5+Paytable!E4*I5+Paytable!F4*J5</f>
-        <v>0.00561912380568425</v>
+        <v>0.00555911355274599</v>
       </c>
       <c r="L5" s="30" t="n">
         <f aca="false">IF($K$12=0,0,K5/$K$12)</f>
-        <v>0.0209204395190634</v>
+        <v>0.0209359889938215</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5185,43 +5185,43 @@
       </c>
       <c r="C6" s="36" t="n">
         <f aca="false">Poids!I6</f>
-        <v>0.0770416024653313</v>
+        <v>0.0767787067053404</v>
       </c>
       <c r="D6" s="36" t="n">
         <f aca="false">Poids!J6</f>
-        <v>0.0783512178504514</v>
+        <v>0.0780852147343405</v>
       </c>
       <c r="E6" s="36" t="n">
         <f aca="false">Poids!K6</f>
-        <v>0.0809307030854831</v>
+        <v>0.0806587128213746</v>
       </c>
       <c r="F6" s="36" t="n">
         <f aca="false">Poids!L6</f>
-        <v>0.0831808351355848</v>
+        <v>0.082904990880451</v>
       </c>
       <c r="G6" s="36" t="n">
         <f aca="false">Poids!M6</f>
-        <v>0.0853718601214907</v>
+        <v>0.0850924562264769</v>
       </c>
       <c r="H6" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C6*D6*E6*(1-F6)^NB_LIGNES,NB_PAYLINES*C6*D6*E6*(1-F6))</f>
-        <v>0.00895773171013786</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C6*D6*E6*((1-NB_LIGNES*Poids!$L$12)*(1-F6/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F6/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C6*D6*E6*(1-F6))</f>
+        <v>0.00886962409084453</v>
       </c>
       <c r="I6" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C6*D6*E6*F6*(1-G6)^NB_LIGNES,NB_PAYLINES*C6*D6*E6*F6*(1-G6))</f>
-        <v>0.000743330928286529</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C6*D6*E6*F6*((1-NB_LIGNES*Poids!$M$12)*(1-G6/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G6/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C6*D6*E6*F6*(1-G6))</f>
+        <v>0.000733582172405446</v>
       </c>
       <c r="J6" s="37" t="n">
         <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C6*D6*E6*F6*G6</f>
-        <v>6.93828904521621E-005</v>
+        <v>6.82279967180883E-005</v>
       </c>
       <c r="K6" s="30" t="n">
         <f aca="false">Paytable!D5*H6+Paytable!E5*I6+Paytable!F5*J6</f>
-        <v>0.012114453082758</v>
+        <v>0.0119829856680083</v>
       </c>
       <c r="L6" s="30" t="n">
         <f aca="false">IF($K$12=0,0,K6/$K$12)</f>
-        <v>0.0451030608665346</v>
+        <v>0.045128715878563</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5235,43 +5235,43 @@
       </c>
       <c r="C7" s="36" t="n">
         <f aca="false">Poids!I7</f>
-        <v>0.102722136620442</v>
+        <v>0.102371608940454</v>
       </c>
       <c r="D7" s="36" t="n">
         <f aca="false">Poids!J7</f>
-        <v>0.102197240674502</v>
+        <v>0.10185028008827</v>
       </c>
       <c r="E7" s="36" t="n">
         <f aca="false">Poids!K7</f>
-        <v>0.104535491485416</v>
+        <v>0.104184170727609</v>
       </c>
       <c r="F7" s="36" t="n">
         <f aca="false">Poids!L7</f>
-        <v>0.106471468973548</v>
+        <v>0.106118388326977</v>
       </c>
       <c r="G7" s="36" t="n">
         <f aca="false">Poids!M7</f>
-        <v>0.108356591692661</v>
+        <v>0.108001963672067</v>
       </c>
       <c r="H7" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C7*D7*E7*(1-F7)^NB_LIGNES,NB_PAYLINES*C7*D7*E7*(1-F7))</f>
-        <v>0.0196112555846103</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C7*D7*E7*((1-NB_LIGNES*Poids!$L$12)*(1-F7/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F7/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C7*D7*E7*(1-F7))</f>
+        <v>0.019420190909289</v>
       </c>
       <c r="I7" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C7*D7*E7*F7*(1-G7)^NB_LIGNES,NB_PAYLINES*C7*D7*E7*F7*(1-G7))</f>
-        <v>0.002083633947722</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C7*D7*E7*F7*((1-NB_LIGNES*Poids!$M$12)*(1-G7/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G7/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C7*D7*E7*F7*(1-G7))</f>
+        <v>0.00205649678723198</v>
       </c>
       <c r="J7" s="37" t="n">
         <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C7*D7*E7*F7*G7</f>
-        <v>0.000253212742680265</v>
+        <v>0.000248997959929023</v>
       </c>
       <c r="K7" s="30" t="n">
         <f aca="false">Paytable!D6*H7+Paytable!E6*I7+Paytable!F6*J7</f>
-        <v>0.0216656692374181</v>
+        <v>0.0214299344389512</v>
       </c>
       <c r="L7" s="30" t="n">
         <f aca="false">IF($K$12=0,0,K7/$K$12)</f>
-        <v>0.0806629892124693</v>
+        <v>0.0807065492178298</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5285,43 +5285,43 @@
       </c>
       <c r="C8" s="36" t="n">
         <f aca="false">Poids!I8</f>
-        <v>0.136962848827256</v>
+        <v>0.136495478587272</v>
       </c>
       <c r="D8" s="36" t="n">
         <f aca="false">Poids!J8</f>
-        <v>0.136262987566002</v>
+        <v>0.135800373451027</v>
       </c>
       <c r="E8" s="36" t="n">
         <f aca="false">Poids!K8</f>
-        <v>0.134884505142472</v>
+        <v>0.134431188035624</v>
       </c>
       <c r="F8" s="36" t="n">
         <f aca="false">Poids!L8</f>
-        <v>0.136416569622359</v>
+        <v>0.13596418504394</v>
       </c>
       <c r="G8" s="36" t="n">
         <f aca="false">Poids!M8</f>
-        <v>0.137908389427023</v>
+        <v>0.13745704467354</v>
       </c>
       <c r="H8" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C8*D8*E8*(1-F8)^NB_LIGNES,NB_PAYLINES*C8*D8*E8*(1-F8))</f>
-        <v>0.043478749712825</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C8*D8*E8*((1-NB_LIGNES*Poids!$L$12)*(1-F8/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F8/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C8*D8*E8*(1-F8))</f>
+        <v>0.0430606922131039</v>
       </c>
       <c r="I8" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C8*D8*E8*F8*(1-G8)^NB_LIGNES,NB_PAYLINES*C8*D8*E8*F8*(1-G8))</f>
-        <v>0.00592097584276931</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C8*D8*E8*F8*((1-NB_LIGNES*Poids!$M$12)*(1-G8/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G8/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C8*D8*E8*F8*(1-G8))</f>
+        <v>0.00584459629827535</v>
       </c>
       <c r="J8" s="37" t="n">
         <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C8*D8*E8*F8*G8</f>
-        <v>0.000947175720420152</v>
+        <v>0.000931409768649458</v>
       </c>
       <c r="K8" s="30" t="n">
         <f aca="false">Paytable!D7*H8+Paytable!E7*I8+Paytable!F7*J8</f>
-        <v>0.0375970134570005</v>
+        <v>0.037185643358856</v>
       </c>
       <c r="L8" s="30" t="n">
         <f aca="false">IF($K$12=0,0,K8/$K$12)</f>
-        <v>0.139976635739709</v>
+        <v>0.140043590169987</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5335,43 +5335,43 @@
       </c>
       <c r="C9" s="36" t="n">
         <f aca="false">Poids!I9</f>
-        <v>0.188323917137476</v>
+        <v>0.187681283057499</v>
       </c>
       <c r="D9" s="36" t="n">
         <f aca="false">Poids!J9</f>
-        <v>0.187361607903253</v>
+        <v>0.186725513495162</v>
       </c>
       <c r="E9" s="36" t="n">
         <f aca="false">Poids!K9</f>
-        <v>0.185466194570899</v>
+        <v>0.184842883548983</v>
       </c>
       <c r="F9" s="36" t="n">
         <f aca="false">Poids!L9</f>
-        <v>0.182997837298286</v>
+        <v>0.182390979936992</v>
       </c>
       <c r="G9" s="36" t="n">
         <f aca="false">Poids!M9</f>
-        <v>0.180594319487769</v>
+        <v>0.180003272786778</v>
       </c>
       <c r="H9" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C9*D9*E9*(1-F9)^NB_LIGNES,NB_PAYLINES*C9*D9*E9*(1-F9))</f>
-        <v>0.106931103008294</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C9*D9*E9*((1-NB_LIGNES*Poids!$L$12)*(1-F9/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F9/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C9*D9*E9*(1-F9))</f>
+        <v>0.105926111743055</v>
       </c>
       <c r="I9" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C9*D9*E9*F9*(1-G9)^NB_LIGNES,NB_PAYLINES*C9*D9*E9*F9*(1-G9))</f>
-        <v>0.0196257276626507</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C9*D9*E9*F9*((1-NB_LIGNES*Poids!$M$12)*(1-G9/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G9/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C9*D9*E9*F9*(1-G9))</f>
+        <v>0.0193763884508822</v>
       </c>
       <c r="J9" s="37" t="n">
         <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C9*D9*E9*F9*G9</f>
-        <v>0.00432544588838225</v>
+        <v>0.00425344787387156</v>
       </c>
       <c r="K9" s="30" t="n">
         <f aca="false">Paytable!D8*H9+Paytable!E8*I9+Paytable!F8*J9</f>
-        <v>0.0572958939870496</v>
+        <v>0.0566365296061398</v>
       </c>
       <c r="L9" s="30" t="n">
         <f aca="false">IF($K$12=0,0,K9/$K$12)</f>
-        <v>0.213317116030473</v>
+        <v>0.213296913119661</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5385,43 +5385,43 @@
       </c>
       <c r="C10" s="36" t="n">
         <f aca="false">Poids!I10</f>
-        <v>0.205444273240883</v>
+        <v>0.204743217880908</v>
       </c>
       <c r="D10" s="36" t="n">
         <f aca="false">Poids!J10</f>
-        <v>0.204394481349004</v>
+        <v>0.20370056017654</v>
       </c>
       <c r="E10" s="36" t="n">
         <f aca="false">Poids!K10</f>
-        <v>0.202326757713708</v>
+        <v>0.201646782053436</v>
       </c>
       <c r="F10" s="36" t="n">
         <f aca="false">Poids!L10</f>
-        <v>0.199634004325403</v>
+        <v>0.198971978113082</v>
       </c>
       <c r="G10" s="36" t="n">
         <f aca="false">Poids!M10</f>
-        <v>0.197011984895748</v>
+        <v>0.196367206676485</v>
       </c>
       <c r="H10" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C10*D10*E10*(1-F10)^NB_LIGNES,NB_PAYLINES*C10*D10*E10*(1-F10))</f>
-        <v>0.135998823720064</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C10*D10*E10*((1-NB_LIGNES*Poids!$L$12)*(1-F10/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F10/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C10*D10*E10*(1-F10))</f>
+        <v>0.134731997462115</v>
       </c>
       <c r="I10" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C10*D10*E10*F10*(1-G10)^NB_LIGNES,NB_PAYLINES*C10*D10*E10*F10*(1-G10))</f>
-        <v>0.027238933822196</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C10*D10*E10*F10*((1-NB_LIGNES*Poids!$M$12)*(1-G10/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G10/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C10*D10*E10*F10*(1-G10))</f>
+        <v>0.0268950655691664</v>
       </c>
       <c r="J10" s="37" t="n">
         <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C10*D10*E10*F10*G10</f>
-        <v>0.00668303426428853</v>
+        <v>0.00657179366381586</v>
       </c>
       <c r="K10" s="30" t="n">
         <f aca="false">Paytable!D9*H10+Paytable!E9*I10+Paytable!F9*J10</f>
-        <v>0.0644281178548437</v>
+        <v>0.0636815944924321</v>
       </c>
       <c r="L10" s="30" t="n">
         <f aca="false">IF($K$12=0,0,K10/$K$12)</f>
-        <v>0.239870945990879</v>
+        <v>0.239829093029409</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5435,43 +5435,43 @@
       </c>
       <c r="C11" s="36" t="n">
         <f aca="false">Poids!I11</f>
-        <v>0.22256462934429</v>
+        <v>0.221805152704317</v>
       </c>
       <c r="D11" s="36" t="n">
         <f aca="false">Poids!J11</f>
-        <v>0.221427354794754</v>
+        <v>0.220675606857919</v>
       </c>
       <c r="E11" s="36" t="n">
         <f aca="false">Poids!K11</f>
-        <v>0.219187320856517</v>
+        <v>0.218450680557889</v>
       </c>
       <c r="F11" s="36" t="n">
         <f aca="false">Poids!L11</f>
-        <v>0.21627017135252</v>
+        <v>0.215552976289173</v>
       </c>
       <c r="G11" s="36" t="n">
         <f aca="false">Poids!M11</f>
-        <v>0.213429650303727</v>
+        <v>0.212731140566192</v>
       </c>
       <c r="H11" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C11*D11*E11*(1-F11)^NB_LIGNES,NB_PAYLINES*C11*D11*E11*(1-F11))</f>
-        <v>0.169316474955139</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C11*D11*E11*((1-NB_LIGNES*Poids!$L$12)*(1-F11/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F11/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C11*D11*E11*(1-F11))</f>
+        <v>0.167754036041489</v>
       </c>
       <c r="I11" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C11*D11*E11*F11*(1-G11)^NB_LIGNES,NB_PAYLINES*C11*D11*E11*F11*(1-G11))</f>
-        <v>0.0367508203331024</v>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C11*D11*E11*F11*((1-NB_LIGNES*Poids!$M$12)*(1-G11/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G11/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C11*D11*E11*F11*(1-G11))</f>
+        <v>0.036289957135012</v>
       </c>
       <c r="J11" s="37" t="n">
         <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C11*D11*E11*F11*G11</f>
-        <v>0.00997204475746881</v>
+        <v>0.00980605784151228</v>
       </c>
       <c r="K11" s="30" t="n">
         <f aca="false">Paytable!D10*H11+Paytable!E10*I11+Paytable!F10*J11</f>
-        <v>0.0698746498513456</v>
+        <v>0.0690532624674223</v>
       </c>
       <c r="L11" s="30" t="n">
         <f aca="false">IF($K$12=0,0,K11/$K$12)</f>
-        <v>0.260148812640871</v>
+        <v>0.26005914959073</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5485,19 +5485,19 @@
       <c r="G12" s="34"/>
       <c r="H12" s="38" t="n">
         <f aca="false">SUM(H5:H11)</f>
-        <v>0.487311529161592</v>
+        <v>0.482750096439595</v>
       </c>
       <c r="I12" s="38" t="n">
         <f aca="false">SUM(I5:I11)</f>
-        <v>0.0925436546888427</v>
+        <v>0.0913739392299969</v>
       </c>
       <c r="J12" s="38" t="n">
         <f aca="false">SUM(J5:J11)</f>
-        <v>0.0222622885973998</v>
+        <v>0.0218917278231263</v>
       </c>
       <c r="K12" s="33" t="n">
         <f aca="false">SUM(K5:K11)</f>
-        <v>0.2685949212761</v>
+        <v>0.265529063584556</v>
       </c>
       <c r="L12" s="33" t="n">
         <f aca="false">SUM(L5:L11)</f>
@@ -5577,11 +5577,11 @@
         <v>0.0684373472380642</v>
       </c>
       <c r="H17" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C17*D17*E17*(1-F17)^NB_LIGNES,NB_PAYLINES*C17*D17*E17*(1-F17))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C17*D17*E17*((1-NB_LIGNES*Poids!$L$26)*(1-F17/(1-Poids!$L$26))^NB_LIGNES+NB_LIGNES*Poids!$L$26*(1-F17/(1-Poids!$L$26))^(NB_LIGNES-1)),NB_PAYLINES*C17*D17*E17*(1-F17))</f>
         <v>0.00422298499443559</v>
       </c>
       <c r="I17" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C17*D17*E17*F17*(1-G17)^NB_LIGNES,NB_PAYLINES*C17*D17*E17*F17*(1-G17))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C17*D17*E17*F17*((1-NB_LIGNES*Poids!$M$26)*(1-G17/(1-Poids!$M$26))^NB_LIGNES+NB_LIGNES*Poids!$M$26*(1-G17/(1-Poids!$M$26))^(NB_LIGNES-1)),NB_PAYLINES*C17*D17*E17*F17*(1-G17))</f>
         <v>0.000278166880253863</v>
       </c>
       <c r="J17" s="37" t="n">
@@ -5627,11 +5627,11 @@
         <v>0.0912497963174189</v>
       </c>
       <c r="H18" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C18*D18*E18*(1-F18)^NB_LIGNES,NB_PAYLINES*C18*D18*E18*(1-F18))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C18*D18*E18*((1-NB_LIGNES*Poids!$L$26)*(1-F18/(1-Poids!$L$26))^NB_LIGNES+NB_LIGNES*Poids!$L$26*(1-F18/(1-Poids!$L$26))^(NB_LIGNES-1)),NB_PAYLINES*C18*D18*E18*(1-F18))</f>
         <v>0.0110506014096863</v>
       </c>
       <c r="I18" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C18*D18*E18*F18*(1-G18)^NB_LIGNES,NB_PAYLINES*C18*D18*E18*F18*(1-G18))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C18*D18*E18*F18*((1-NB_LIGNES*Poids!$M$26)*(1-G18/(1-Poids!$M$26))^NB_LIGNES+NB_LIGNES*Poids!$M$26*(1-G18/(1-Poids!$M$26))^(NB_LIGNES-1)),NB_PAYLINES*C18*D18*E18*F18*(1-G18))</f>
         <v>0.000982926879138738</v>
       </c>
       <c r="J18" s="37" t="n">
@@ -5677,11 +5677,11 @@
         <v>0.114062245396774</v>
       </c>
       <c r="H19" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C19*D19*E19*(1-F19)^NB_LIGNES,NB_PAYLINES*C19*D19*E19*(1-F19))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C19*D19*E19*((1-NB_LIGNES*Poids!$L$26)*(1-F19/(1-Poids!$L$26))^NB_LIGNES+NB_LIGNES*Poids!$L$26*(1-F19/(1-Poids!$L$26))^(NB_LIGNES-1)),NB_PAYLINES*C19*D19*E19*(1-F19))</f>
         <v>0.0226008087661245</v>
       </c>
       <c r="I19" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C19*D19*E19*F19*(1-G19)^NB_LIGNES,NB_PAYLINES*C19*D19*E19*F19*(1-G19))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C19*D19*E19*F19*((1-NB_LIGNES*Poids!$M$26)*(1-G19/(1-Poids!$M$26))^NB_LIGNES+NB_LIGNES*Poids!$M$26*(1-G19/(1-Poids!$M$26))^(NB_LIGNES-1)),NB_PAYLINES*C19*D19*E19*F19*(1-G19))</f>
         <v>0.00253218870074847</v>
       </c>
       <c r="J19" s="37" t="n">
@@ -5727,11 +5727,11 @@
         <v>0.140133615773179</v>
       </c>
       <c r="H20" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C20*D20*E20*(1-F20)^NB_LIGNES,NB_PAYLINES*C20*D20*E20*(1-F20))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C20*D20*E20*((1-NB_LIGNES*Poids!$L$26)*(1-F20/(1-Poids!$L$26))^NB_LIGNES+NB_LIGNES*Poids!$L$26*(1-F20/(1-Poids!$L$26))^(NB_LIGNES-1)),NB_PAYLINES*C20*D20*E20*(1-F20))</f>
         <v>0.0439423226061669</v>
       </c>
       <c r="I20" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C20*D20*E20*F20*(1-G20)^NB_LIGNES,NB_PAYLINES*C20*D20*E20*F20*(1-G20))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C20*D20*E20*F20*((1-NB_LIGNES*Poids!$M$26)*(1-G20/(1-Poids!$M$26))^NB_LIGNES+NB_LIGNES*Poids!$M$26*(1-G20/(1-Poids!$M$26))^(NB_LIGNES-1)),NB_PAYLINES*C20*D20*E20*F20*(1-G20))</f>
         <v>0.00608376497705008</v>
       </c>
       <c r="J20" s="37" t="n">
@@ -5777,11 +5777,11 @@
         <v>0.171093368095161</v>
       </c>
       <c r="H21" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C21*D21*E21*(1-F21)^NB_LIGNES,NB_PAYLINES*C21*D21*E21*(1-F21))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C21*D21*E21*((1-NB_LIGNES*Poids!$L$26)*(1-F21/(1-Poids!$L$26))^NB_LIGNES+NB_LIGNES*Poids!$L$26*(1-F21/(1-Poids!$L$26))^(NB_LIGNES-1)),NB_PAYLINES*C21*D21*E21*(1-F21))</f>
         <v>0.0930280320205477</v>
       </c>
       <c r="I21" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C21*D21*E21*F21*(1-G21)^NB_LIGNES,NB_PAYLINES*C21*D21*E21*F21*(1-G21))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C21*D21*E21*F21*((1-NB_LIGNES*Poids!$M$26)*(1-G21/(1-Poids!$M$26))^NB_LIGNES+NB_LIGNES*Poids!$M$26*(1-G21/(1-Poids!$M$26))^(NB_LIGNES-1)),NB_PAYLINES*C21*D21*E21*F21*(1-G21))</f>
         <v>0.0161707869641766</v>
       </c>
       <c r="J21" s="37" t="n">
@@ -5827,11 +5827,11 @@
         <v>0.187387974580414</v>
       </c>
       <c r="H22" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C22*D22*E22*(1-F22)^NB_LIGNES,NB_PAYLINES*C22*D22*E22*(1-F22))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C22*D22*E22*((1-NB_LIGNES*Poids!$L$26)*(1-F22/(1-Poids!$L$26))^NB_LIGNES+NB_LIGNES*Poids!$L$26*(1-F22/(1-Poids!$L$26))^(NB_LIGNES-1)),NB_PAYLINES*C22*D22*E22*(1-F22))</f>
         <v>0.119778239109449</v>
       </c>
       <c r="I22" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C22*D22*E22*F22*(1-G22)^NB_LIGNES,NB_PAYLINES*C22*D22*E22*F22*(1-G22))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C22*D22*E22*F22*((1-NB_LIGNES*Poids!$M$26)*(1-G22/(1-Poids!$M$26))^NB_LIGNES+NB_LIGNES*Poids!$M$26*(1-G22/(1-Poids!$M$26))^(NB_LIGNES-1)),NB_PAYLINES*C22*D22*E22*F22*(1-G22))</f>
         <v>0.0228109278798673</v>
       </c>
       <c r="J22" s="37" t="n">
@@ -5877,11 +5877,11 @@
         <v>0.203682581065667</v>
       </c>
       <c r="H23" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C23*D23*E23*(1-F23)^NB_LIGNES,NB_PAYLINES*C23*D23*E23*(1-F23))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^3*C23*D23*E23*((1-NB_LIGNES*Poids!$L$26)*(1-F23/(1-Poids!$L$26))^NB_LIGNES+NB_LIGNES*Poids!$L$26*(1-F23/(1-Poids!$L$26))^(NB_LIGNES-1)),NB_PAYLINES*C23*D23*E23*(1-F23))</f>
         <v>0.150685861789895</v>
       </c>
       <c r="I23" s="37" t="n">
-        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C23*D23*E23*F23*(1-G23)^NB_LIGNES,NB_PAYLINES*C23*D23*E23*F23*(1-G23))</f>
+        <f aca="false">IF(MODE_GAIN="WAYS",NB_LIGNES^4*C23*D23*E23*F23*((1-NB_LIGNES*Poids!$M$26)*(1-G23/(1-Poids!$M$26))^NB_LIGNES+NB_LIGNES*Poids!$M$26*(1-G23/(1-Poids!$M$26))^(NB_LIGNES-1)),NB_PAYLINES*C23*D23*E23*F23*(1-G23))</f>
         <v>0.0312028751119265</v>
       </c>
       <c r="J23" s="37" t="n">
@@ -5999,23 +5999,23 @@
       </c>
       <c r="B5" s="39" t="n">
         <f aca="false">Poids!I12</f>
-        <v>0.0154083204930663</v>
+        <v>0.0187681283057499</v>
       </c>
       <c r="C5" s="39" t="n">
         <f aca="false">Poids!J12</f>
-        <v>0.0153295861011753</v>
+        <v>0.0186725513495162</v>
       </c>
       <c r="D5" s="39" t="n">
         <f aca="false">Poids!K12</f>
-        <v>0.0151745068285281</v>
+        <v>0.0184842883548983</v>
       </c>
       <c r="E5" s="39" t="n">
         <f aca="false">Poids!L12</f>
-        <v>0.0149725503244053</v>
+        <v>0.0182390979936992</v>
       </c>
       <c r="F5" s="39" t="n">
         <f aca="false">Poids!M12</f>
-        <v>0.0147758988671811</v>
+        <v>0.0180003272786778</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6049,23 +6049,23 @@
       </c>
       <c r="B7" s="39" t="n">
         <f aca="false">Poids!I13</f>
-        <v>0.00017120356103407</v>
+        <v>0.00017061934823409</v>
       </c>
       <c r="C7" s="39" t="n">
         <f aca="false">Poids!J13</f>
-        <v>0.000170328734457503</v>
+        <v>0.000169750466813784</v>
       </c>
       <c r="D7" s="39" t="n">
         <f aca="false">Poids!K13</f>
-        <v>0.00016860563142809</v>
+        <v>0.00016803898504453</v>
       </c>
       <c r="E7" s="39" t="n">
         <f aca="false">Poids!L13</f>
-        <v>0.00016636167027117</v>
+        <v>0.000165809981760902</v>
       </c>
       <c r="F7" s="39" t="n">
         <f aca="false">Poids!M13</f>
-        <v>0.00016417665407979</v>
+        <v>0.000163639338897071</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6123,24 +6123,24 @@
         <v>0</v>
       </c>
       <c r="B12" s="41" t="n">
-        <f aca="false">IF($A12&gt;NB_LIGNES,0,BINOMDIST($A12,NB_LIGNES,B$5,FALSE()))</f>
-        <v>0.925296260032285</v>
+        <f aca="false">IF($A12=0,1-NB_LIGNES*B$5,IF($A12=1,NB_LIGNES*B$5,0))</f>
+        <v>0.906159358471251</v>
       </c>
       <c r="C12" s="41" t="n">
-        <f aca="false">IF($A12&gt;NB_LIGNES,0,BINOMDIST($A12,NB_LIGNES,C$5,FALSE()))</f>
-        <v>0.92566628291765</v>
+        <f aca="false">IF($A12=0,1-NB_LIGNES*C$5,IF($A12=1,NB_LIGNES*C$5,0))</f>
+        <v>0.906637243252419</v>
       </c>
       <c r="D12" s="41" t="n">
-        <f aca="false">IF($A12&gt;NB_LIGNES,0,BINOMDIST($A12,NB_LIGNES,D$5,FALSE()))</f>
-        <v>0.926395445061109</v>
+        <f aca="false">IF($A12=0,1-NB_LIGNES*D$5,IF($A12=1,NB_LIGNES*D$5,0))</f>
+        <v>0.907578558225508</v>
       </c>
       <c r="E12" s="41" t="n">
-        <f aca="false">IF($A12&gt;NB_LIGNES,0,BINOMDIST($A12,NB_LIGNES,E$5,FALSE()))</f>
-        <v>0.927345706481366</v>
+        <f aca="false">IF($A12=0,1-NB_LIGNES*E$5,IF($A12=1,NB_LIGNES*E$5,0))</f>
+        <v>0.908804510031504</v>
       </c>
       <c r="F12" s="41" t="n">
-        <f aca="false">IF($A12&gt;NB_LIGNES,0,BINOMDIST($A12,NB_LIGNES,F$5,FALSE()))</f>
-        <v>0.928271755362511</v>
+        <f aca="false">IF($A12=0,1-NB_LIGNES*F$5,IF($A12=1,NB_LIGNES*F$5,0))</f>
+        <v>0.909998363606611</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6148,24 +6148,24 @@
         <v>1</v>
       </c>
       <c r="B13" s="41" t="n">
-        <f aca="false">IF($A13&gt;NB_LIGNES,0,BINOMDIST($A13,NB_LIGNES,B$5,FALSE()))</f>
-        <v>0.0724018982810865</v>
+        <f aca="false">IF($A13=0,1-NB_LIGNES*B$5,IF($A13=1,NB_LIGNES*B$5,0))</f>
+        <v>0.0938406415287494</v>
       </c>
       <c r="C13" s="41" t="n">
-        <f aca="false">IF($A13&gt;NB_LIGNES,0,BINOMDIST($A13,NB_LIGNES,C$5,FALSE()))</f>
-        <v>0.0720549779126349</v>
+        <f aca="false">IF($A13=0,1-NB_LIGNES*C$5,IF($A13=1,NB_LIGNES*C$5,0))</f>
+        <v>0.093362756747581</v>
       </c>
       <c r="D13" s="41" t="n">
-        <f aca="false">IF($A13&gt;NB_LIGNES,0,BINOMDIST($A13,NB_LIGNES,D$5,FALSE()))</f>
-        <v>0.0713709896040916</v>
+        <f aca="false">IF($A13=0,1-NB_LIGNES*D$5,IF($A13=1,NB_LIGNES*D$5,0))</f>
+        <v>0.0924214417744917</v>
       </c>
       <c r="E13" s="41" t="n">
-        <f aca="false">IF($A13&gt;NB_LIGNES,0,BINOMDIST($A13,NB_LIGNES,E$5,FALSE()))</f>
-        <v>0.0704789001716964</v>
+        <f aca="false">IF($A13=0,1-NB_LIGNES*E$5,IF($A13=1,NB_LIGNES*E$5,0))</f>
+        <v>0.0911954899684961</v>
       </c>
       <c r="F13" s="41" t="n">
-        <f aca="false">IF($A13&gt;NB_LIGNES,0,BINOMDIST($A13,NB_LIGNES,F$5,FALSE()))</f>
-        <v>0.0696087801888235</v>
+        <f aca="false">IF($A13=0,1-NB_LIGNES*F$5,IF($A13=1,NB_LIGNES*F$5,0))</f>
+        <v>0.090001636393389</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6173,24 +6173,24 @@
         <v>2</v>
       </c>
       <c r="B14" s="41" t="n">
-        <f aca="false">IF($A14&gt;NB_LIGNES,0,BINOMDIST($A14,NB_LIGNES,B$5,FALSE()))</f>
-        <v>0.00226610010269441</v>
+        <f aca="false">IF($A14=0,1-NB_LIGNES*B$5,IF($A14=1,NB_LIGNES*B$5,0))</f>
+        <v>0</v>
       </c>
       <c r="C14" s="41" t="n">
-        <f aca="false">IF($A14&gt;NB_LIGNES,0,BINOMDIST($A14,NB_LIGNES,C$5,FALSE()))</f>
-        <v>0.00224353849234982</v>
+        <f aca="false">IF($A14=0,1-NB_LIGNES*C$5,IF($A14=1,NB_LIGNES*C$5,0))</f>
+        <v>0</v>
       </c>
       <c r="D14" s="41" t="n">
-        <f aca="false">IF($A14&gt;NB_LIGNES,0,BINOMDIST($A14,NB_LIGNES,D$5,FALSE()))</f>
-        <v>0.00219941416345429</v>
+        <f aca="false">IF($A14=0,1-NB_LIGNES*D$5,IF($A14=1,NB_LIGNES*D$5,0))</f>
+        <v>0</v>
       </c>
       <c r="E14" s="41" t="n">
-        <f aca="false">IF($A14&gt;NB_LIGNES,0,BINOMDIST($A14,NB_LIGNES,E$5,FALSE()))</f>
-        <v>0.00214257761035389</v>
+        <f aca="false">IF($A14=0,1-NB_LIGNES*E$5,IF($A14=1,NB_LIGNES*E$5,0))</f>
+        <v>0</v>
       </c>
       <c r="F14" s="41" t="n">
-        <f aca="false">IF($A14&gt;NB_LIGNES,0,BINOMDIST($A14,NB_LIGNES,F$5,FALSE()))</f>
-        <v>0.00208791541976141</v>
+        <f aca="false">IF($A14=0,1-NB_LIGNES*F$5,IF($A14=1,NB_LIGNES*F$5,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6198,24 +6198,24 @@
         <v>3</v>
       </c>
       <c r="B15" s="41" t="n">
-        <f aca="false">IF($A15&gt;NB_LIGNES,0,BINOMDIST($A15,NB_LIGNES,B$5,FALSE()))</f>
-        <v>3.54632253942788E-005</v>
+        <f aca="false">IF($A15=0,1-NB_LIGNES*B$5,IF($A15=1,NB_LIGNES*B$5,0))</f>
+        <v>0</v>
       </c>
       <c r="C15" s="41" t="n">
-        <f aca="false">IF($A15&gt;NB_LIGNES,0,BINOMDIST($A15,NB_LIGNES,C$5,FALSE()))</f>
-        <v>3.49279474678228E-005</v>
+        <f aca="false">IF($A15=0,1-NB_LIGNES*C$5,IF($A15=1,NB_LIGNES*C$5,0))</f>
+        <v>0</v>
       </c>
       <c r="D15" s="41" t="n">
-        <f aca="false">IF($A15&gt;NB_LIGNES,0,BINOMDIST($A15,NB_LIGNES,D$5,FALSE()))</f>
-        <v>3.38892783274929E-005</v>
+        <f aca="false">IF($A15=0,1-NB_LIGNES*D$5,IF($A15=1,NB_LIGNES*D$5,0))</f>
+        <v>0</v>
       </c>
       <c r="E15" s="41" t="n">
-        <f aca="false">IF($A15&gt;NB_LIGNES,0,BINOMDIST($A15,NB_LIGNES,E$5,FALSE()))</f>
-        <v>3.25674691659939E-005</v>
+        <f aca="false">IF($A15=0,1-NB_LIGNES*E$5,IF($A15=1,NB_LIGNES*E$5,0))</f>
+        <v>0</v>
       </c>
       <c r="F15" s="41" t="n">
-        <f aca="false">IF($A15&gt;NB_LIGNES,0,BINOMDIST($A15,NB_LIGNES,F$5,FALSE()))</f>
-        <v>3.13135123776916E-005</v>
+        <f aca="false">IF($A15=0,1-NB_LIGNES*F$5,IF($A15=1,NB_LIGNES*F$5,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6223,24 +6223,24 @@
         <v>4</v>
       </c>
       <c r="B16" s="41" t="n">
-        <f aca="false">IF($A16&gt;NB_LIGNES,0,BINOMDIST($A16,NB_LIGNES,B$5,FALSE()))</f>
-        <v>2.77490026559302E-007</v>
+        <f aca="false">IF($A16=0,1-NB_LIGNES*B$5,IF($A16=1,NB_LIGNES*B$5,0))</f>
+        <v>0</v>
       </c>
       <c r="C16" s="41" t="n">
-        <f aca="false">IF($A16&gt;NB_LIGNES,0,BINOMDIST($A16,NB_LIGNES,C$5,FALSE()))</f>
-        <v>2.71883348218652E-007</v>
+        <f aca="false">IF($A16=0,1-NB_LIGNES*C$5,IF($A16=1,NB_LIGNES*C$5,0))</f>
+        <v>0</v>
       </c>
       <c r="D16" s="41" t="n">
-        <f aca="false">IF($A16&gt;NB_LIGNES,0,BINOMDIST($A16,NB_LIGNES,D$5,FALSE()))</f>
-        <v>2.61088430874367E-007</v>
+        <f aca="false">IF($A16=0,1-NB_LIGNES*D$5,IF($A16=1,NB_LIGNES*D$5,0))</f>
+        <v>0</v>
       </c>
       <c r="E16" s="41" t="n">
-        <f aca="false">IF($A16&gt;NB_LIGNES,0,BINOMDIST($A16,NB_LIGNES,E$5,FALSE()))</f>
-        <v>2.47514965794583E-007</v>
+        <f aca="false">IF($A16=0,1-NB_LIGNES*E$5,IF($A16=1,NB_LIGNES*E$5,0))</f>
+        <v>0</v>
       </c>
       <c r="F16" s="41" t="n">
-        <f aca="false">IF($A16&gt;NB_LIGNES,0,BINOMDIST($A16,NB_LIGNES,F$5,FALSE()))</f>
-        <v>2.34812207464776E-007</v>
+        <f aca="false">IF($A16=0,1-NB_LIGNES*F$5,IF($A16=1,NB_LIGNES*F$5,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6248,24 +6248,24 @@
         <v>5</v>
       </c>
       <c r="B17" s="41" t="n">
-        <f aca="false">IF($A17&gt;NB_LIGNES,0,BINOMDIST($A17,NB_LIGNES,B$5,FALSE()))</f>
-        <v>8.68513385162134E-010</v>
+        <f aca="false">IF($A17=0,1-NB_LIGNES*B$5,IF($A17=1,NB_LIGNES*B$5,0))</f>
+        <v>0</v>
       </c>
       <c r="C17" s="41" t="n">
-        <f aca="false">IF($A17&gt;NB_LIGNES,0,BINOMDIST($A17,NB_LIGNES,C$5,FALSE()))</f>
-        <v>8.46549086306129E-010</v>
+        <f aca="false">IF($A17=0,1-NB_LIGNES*C$5,IF($A17=1,NB_LIGNES*C$5,0))</f>
+        <v>0</v>
       </c>
       <c r="D17" s="41" t="n">
-        <f aca="false">IF($A17&gt;NB_LIGNES,0,BINOMDIST($A17,NB_LIGNES,D$5,FALSE()))</f>
-        <v>8.04586843988805E-010</v>
+        <f aca="false">IF($A17=0,1-NB_LIGNES*D$5,IF($A17=1,NB_LIGNES*D$5,0))</f>
+        <v>0</v>
       </c>
       <c r="E17" s="41" t="n">
-        <f aca="false">IF($A17&gt;NB_LIGNES,0,BINOMDIST($A17,NB_LIGNES,E$5,FALSE()))</f>
-        <v>7.52452184479393E-010</v>
+        <f aca="false">IF($A17=0,1-NB_LIGNES*E$5,IF($A17=1,NB_LIGNES*E$5,0))</f>
+        <v>0</v>
       </c>
       <c r="F17" s="41" t="n">
-        <f aca="false">IF($A17&gt;NB_LIGNES,0,BINOMDIST($A17,NB_LIGNES,F$5,FALSE()))</f>
-        <v>7.04319235855019E-010</v>
+        <f aca="false">IF($A17=0,1-NB_LIGNES*F$5,IF($A17=1,NB_LIGNES*F$5,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6308,30 +6308,30 @@
       </c>
       <c r="B21" s="41" t="n">
         <f aca="false">B12</f>
-        <v>0.925296260032285</v>
+        <v>0.906159358471251</v>
       </c>
       <c r="C21" s="41" t="n">
         <f aca="false">C$12*B21</f>
-        <v>0.856515549621689</v>
+        <v>0.821557822711755</v>
       </c>
       <c r="D21" s="41" t="n">
         <f aca="false">D$12*C21</f>
-        <v>0.793472103793545</v>
+        <v>0.745628264235623</v>
       </c>
       <c r="E21" s="41" t="n">
         <f aca="false">E$12*D21</f>
-        <v>0.73582294866568</v>
+        <v>0.677630329344296</v>
       </c>
       <c r="F21" s="41" t="n">
         <f aca="false">F$12*E21</f>
-        <v>0.68304366019391</v>
+        <v>0.616642490833518</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>193</v>
       </c>
       <c r="I21" s="42" t="n">
         <f aca="false">SUMPRODUCT(--($A$21:$A$46&gt;=SCATTER_MIN),$F$21:$F$46)</f>
-        <v>0.0062124527590887</v>
+        <v>0.00678528899288191</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6340,30 +6340,30 @@
       </c>
       <c r="B22" s="41" t="n">
         <f aca="false">B13</f>
-        <v>0.0724018982810865</v>
+        <v>0.0938406415287494</v>
       </c>
       <c r="C22" s="41" t="n">
         <f aca="false">C$12*B22+C$13*B21</f>
-        <v>0.133692197637305</v>
+        <v>0.169680956300159</v>
       </c>
       <c r="D22" s="41" t="n">
         <f aca="false">D$12*C22+D$13*C21</f>
-        <v>0.184982205319201</v>
+        <v>0.229928356153357</v>
       </c>
       <c r="E22" s="41" t="n">
         <f aca="false">E$12*D22+E$13*D21</f>
-        <v>0.227465495070507</v>
+        <v>0.276957861947627</v>
       </c>
       <c r="F22" s="41" t="n">
         <f aca="false">F$12*E22+F$13*E21</f>
-        <v>0.262369532285063</v>
+        <v>0.313019039671104</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>38</v>
       </c>
       <c r="I22" s="40" t="n">
         <f aca="false">IF(I21=0,"-",1/I21)</f>
-        <v>160.967018789321</v>
+        <v>147.377657908019</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6372,23 +6372,23 @@
       </c>
       <c r="B23" s="41" t="n">
         <f aca="false">B14</f>
-        <v>0.00226610010269441</v>
+        <v>0</v>
       </c>
       <c r="C23" s="41" t="n">
         <f aca="false">C$12*B23+C$13*B22+C$14*B21</f>
-        <v>0.00939050741646673</v>
+        <v>0.00876122098808558</v>
       </c>
       <c r="D23" s="41" t="n">
         <f aca="false">D$12*C23+D$13*C22+D$14*C21</f>
-        <v>0.0201249001762044</v>
+        <v>0.023633654935597</v>
       </c>
       <c r="E23" s="41" t="n">
         <f aca="false">E$12*D23+E$13*D22+E$14*D21</f>
-        <v>0.0334001577180299</v>
+        <v>0.0424468012910551</v>
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">F$12*E23+F$13*E22+F$14*E21</f>
-        <v>0.0483743547619385</v>
+        <v>0.0635531805024959</v>
       </c>
       <c r="H23" s="6" t="str">
         <f aca="false">"P(exactement "&amp;Config!A25&amp;" trophées)"</f>
@@ -6396,7 +6396,7 @@
       </c>
       <c r="I23" s="42" t="n">
         <f aca="false">SUMPRODUCT(--($A$21:$A$46=Config!$A$25),$F$21:$F$46)</f>
-        <v>0.00569820294679901</v>
+        <v>0.00645123624721947</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6405,23 +6405,23 @@
       </c>
       <c r="B24" s="41" t="n">
         <f aca="false">B15</f>
-        <v>3.54632253942788E-005</v>
+        <v>0</v>
       </c>
       <c r="C24" s="41" t="n">
         <f aca="false">C$12*B24+C$13*B23+C$14*B22+C$15*B21</f>
-        <v>0.000390866049753853</v>
+        <v>0</v>
       </c>
       <c r="D24" s="41" t="n">
         <f aca="false">D$12*C24+D$13*C23+D$14*C22+D$15*C21</f>
-        <v>0.00135537754219856</v>
+        <v>0.000809724675423806</v>
       </c>
       <c r="E24" s="41" t="n">
         <f aca="false">E$12*D24+E$13*D23+E$14*D22+E$15*D21</f>
-        <v>0.00309746448460835</v>
+        <v>0.00289116417850709</v>
       </c>
       <c r="F24" s="41" t="n">
         <f aca="false">F$12*E24+F$13*E23+F$14*E22+F$15*E21</f>
-        <v>0.00569820294679901</v>
+        <v>0.00645123624721947</v>
       </c>
       <c r="H24" s="6" t="str">
         <f aca="false">"P(exactement "&amp;Config!A26&amp;" trophées)"</f>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="I24" s="42" t="n">
         <f aca="false">SUMPRODUCT(--($A$21:$A$46=Config!$A$26),$F$21:$F$46)</f>
-        <v>0.000481517810045691</v>
+        <v>0.000327406733359517</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6438,23 +6438,23 @@
       </c>
       <c r="B25" s="41" t="n">
         <f aca="false">B16</f>
-        <v>2.77490026559302E-007</v>
+        <v>0</v>
       </c>
       <c r="C25" s="41" t="n">
         <f aca="false">C$12*B25+C$13*B24+C$14*B23+C$15*B22+C$16*B21</f>
-        <v>1.06766702368444E-005</v>
+        <v>0</v>
       </c>
       <c r="D25" s="41" t="n">
         <f aca="false">D$12*C25+D$13*C24+D$14*C23+D$15*C22+D$16*C21</f>
-        <v>6.31952888600212E-005</v>
+        <v>0</v>
       </c>
       <c r="E25" s="41" t="n">
         <f aca="false">E$12*D25+E$13*D24+E$14*D23+E$15*D22+E$16*D21</f>
-        <v>0.000203469357302525</v>
+        <v>7.38432385148554E-005</v>
       </c>
       <c r="F25" s="41" t="n">
         <f aca="false">F$12*E25+F$13*E24+F$14*E23+F$15*E22+F$16*E21</f>
-        <v>0.000481517810045691</v>
+        <v>0.000327406733359517</v>
       </c>
       <c r="H25" s="6" t="str">
         <f aca="false">"P("&amp;Config!A27&amp;" trophées ou plus)"</f>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="I25" s="42" t="n">
         <f aca="false">SUMPRODUCT(--($A$21:$A$46&gt;=Config!$A$27),$F$21:$F$46)</f>
-        <v>3.27320022440019E-005</v>
+        <v>6.64601230292431E-006</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6471,30 +6471,30 @@
       </c>
       <c r="B26" s="41" t="n">
         <f aca="false">B17</f>
-        <v>8.68513385162134E-010</v>
+        <v>0</v>
       </c>
       <c r="C26" s="41" t="n">
         <f aca="false">C$12*B26+C$13*B25+C$14*B24+C$15*B23+C$16*B22+C$17*B21</f>
-        <v>1.99980007095835E-007</v>
+        <v>0</v>
       </c>
       <c r="D26" s="41" t="n">
         <f aca="false">D$12*C26+D$13*C25+D$14*C24+D$15*C23+D$16*C22+D$17*C21</f>
-        <v>2.16077356071625E-006</v>
+        <v>0</v>
       </c>
       <c r="E26" s="41" t="n">
         <f aca="false">E$12*D26+E$13*D25+E$14*D24+E$15*D23+E$16*D22+E$17*D21</f>
-        <v>1.0063520094584E-005</v>
+        <v>0</v>
       </c>
       <c r="F26" s="41" t="n">
         <f aca="false">F$12*E26+F$13*E25+F$14*E24+F$15*E23+F$16*E22+F$17*E21</f>
-        <v>3.1071985271932E-005</v>
+        <v>6.64601230292431E-006</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>194</v>
       </c>
       <c r="I26" s="43" t="n">
         <f aca="false">IF(I21=0,0,(I23*Config!$B$25+I24*Config!$B$26+I25*Config!$B$27)/I21)</f>
-        <v>10.1813608368551</v>
+        <v>10.1014022437298</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6506,19 +6506,19 @@
       </c>
       <c r="C27" s="41" t="n">
         <f aca="false">C$13*B26+C$14*B25+C$15*B24+C$16*B23+C$17*B22</f>
-        <v>2.60120458638045E-009</v>
+        <v>0</v>
       </c>
       <c r="D27" s="41" t="n">
         <f aca="false">D$12*C27+D$13*C26+D$14*C25+D$15*C24+D$16*C23+D$17*C22</f>
-        <v>5.59704230041227E-008</v>
+        <v>0</v>
       </c>
       <c r="E27" s="41" t="n">
         <f aca="false">E$12*D27+E$13*D26+E$14*D25+E$15*D24+E$16*D23+E$17*D22</f>
-        <v>3.88855307090556E-007</v>
+        <v>0</v>
       </c>
       <c r="F27" s="41" t="n">
         <f aca="false">F$12*E27+F$13*E26+F$14*E25+F$15*E24+F$16*E23+F$17*E22</f>
-        <v>1.59129503081093E-006</v>
+        <v>0</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>195</v>
@@ -6537,19 +6537,19 @@
       </c>
       <c r="C28" s="41" t="n">
         <f aca="false">C$14*B26+C$15*B25+C$16*B24+C$17*B23</f>
-        <v>2.32009257114837E-011</v>
+        <v>0</v>
       </c>
       <c r="D28" s="41" t="n">
         <f aca="false">D$12*C28+D$13*C27+D$14*C26+D$15*C25+D$16*C24+D$17*C23</f>
-        <v>1.11841336901251E-009</v>
+        <v>0</v>
       </c>
       <c r="E28" s="41" t="n">
         <f aca="false">E$12*D28+E$13*D27+E$14*D26+E$15*D25+E$16*D24+E$17*D23</f>
-        <v>1.20202446160164E-008</v>
+        <v>0</v>
       </c>
       <c r="F28" s="41" t="n">
         <f aca="false">F$12*E28+F$13*E27+F$14*E26+F$15*E25+F$16*E24+F$17*E23</f>
-        <v>6.63597630337906E-008</v>
+        <v>0</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>196</v>
@@ -6568,26 +6568,26 @@
       </c>
       <c r="C29" s="41" t="n">
         <f aca="false">C$15*B26+C$16*B25+C$17*B24</f>
-        <v>1.35801668465264E-013</v>
+        <v>0</v>
       </c>
       <c r="D29" s="41" t="n">
         <f aca="false">D$12*C29+D$13*C28+D$14*C27+D$15*C26+D$16*C25+D$17*C24</f>
-        <v>1.73820241650843E-011</v>
+        <v>0</v>
       </c>
       <c r="E29" s="41" t="n">
         <f aca="false">E$12*D29+E$13*D28+E$14*D27+E$15*D26+E$16*D25+E$17*D24</f>
-        <v>3.01897227701749E-010</v>
+        <v>0</v>
       </c>
       <c r="F29" s="41" t="n">
         <f aca="false">F$12*E29+F$13*E28+F$14*E27+F$15*E26+F$16*E25+F$17*E24</f>
-        <v>2.29393708032382E-009</v>
+        <v>0</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>197</v>
       </c>
       <c r="I29" s="43" t="n">
         <f aca="false">IF(I28&gt;=1,"Infini (μ ≥ 1)",I26/(1-I28))</f>
-        <v>24.5556276828887</v>
+        <v>24.3627818075392</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6599,19 +6599,19 @@
       </c>
       <c r="C30" s="41" t="n">
         <f aca="false">C$16*B26+C$17*B25</f>
-        <v>4.71043255573437E-016</v>
+        <v>0</v>
       </c>
       <c r="D30" s="41" t="n">
         <f aca="false">D$12*C30+D$13*C29+D$14*C28+D$15*C27+D$16*C26+D$17*C25</f>
-        <v>2.10112837293397E-013</v>
+        <v>0</v>
       </c>
       <c r="E30" s="41" t="n">
         <f aca="false">E$12*D30+E$13*D29+E$14*D28+E$15*D27+E$16*D26+E$17*D25</f>
-        <v>6.22139087953674E-012</v>
+        <v>0</v>
       </c>
       <c r="F30" s="41" t="n">
         <f aca="false">F$12*E30+F$13*E29+F$14*E28+F$15*E27+F$16*E26+F$17*E25</f>
-        <v>6.65698635005767E-011</v>
+        <v>0</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>198</v>
@@ -6630,26 +6630,26 @@
       </c>
       <c r="C31" s="41" t="n">
         <f aca="false">C$17*B26</f>
-        <v>7.35239212653647E-019</v>
+        <v>0</v>
       </c>
       <c r="D31" s="41" t="n">
         <f aca="false">D$12*C31+D$13*C30+D$14*C29+D$15*C28+D$16*C27+D$17*C26</f>
-        <v>1.9592923941008E-015</v>
+        <v>0</v>
       </c>
       <c r="E31" s="41" t="n">
         <f aca="false">E$12*D31+E$13*D30+E$14*D29+E$15*D28+E$16*D27+E$17*D26</f>
-        <v>1.05771087903994E-013</v>
+        <v>0</v>
       </c>
       <c r="F31" s="41" t="n">
         <f aca="false">F$12*E31+F$13*E30+F$14*E29+F$15*E28+F$16*E27+F$17*E26</f>
-        <v>1.63637560293124E-012</v>
+        <v>0</v>
       </c>
       <c r="H31" s="6" t="s">
         <v>199</v>
       </c>
       <c r="I31" s="44" t="n">
         <f aca="false">NB_LIGNES*SUM(B7:F7)</f>
-        <v>0.00420338125635311</v>
+        <v>0.00418929060375188</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6664,22 +6664,22 @@
       </c>
       <c r="D32" s="41" t="n">
         <f aca="false">D$13*C31+D$14*C30+D$15*C29+D$16*C28+D$17*C27</f>
-        <v>1.3841102775637E-017</v>
+        <v>0</v>
       </c>
       <c r="E32" s="41" t="n">
         <f aca="false">E$12*D32+E$13*D31+E$14*D30+E$15*D29+E$16*D28+E$17*D27</f>
-        <v>1.48613497098567E-015</v>
+        <v>0</v>
       </c>
       <c r="F32" s="41" t="n">
         <f aca="false">F$12*E32+F$13*E31+F$14*E30+F$15*E29+F$16*E28+F$17*E27</f>
-        <v>3.42817124979432E-014</v>
+        <v>0</v>
       </c>
       <c r="H32" s="6" t="s">
         <v>200</v>
       </c>
       <c r="I32" s="45" t="n">
         <f aca="false">1-(1-B7)^NB_LIGNES*(1-C7)^NB_LIGNES*(1-D7)^NB_LIGNES*(1-E7)^NB_LIGNES*(1-F7)^NB_LIGNES</f>
-        <v>0.00419491142248873</v>
+        <v>0.00418087742329565</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6694,15 +6694,15 @@
       </c>
       <c r="D33" s="41" t="n">
         <f aca="false">D$14*C31+D$15*C30+D$16*C29+D$17*C28</f>
-        <v>7.17038156557923E-020</v>
+        <v>0</v>
       </c>
       <c r="E33" s="41" t="n">
         <f aca="false">E$12*D33+E$13*D32+E$14*D31+E$15*D30+E$16*D29+E$17*D28</f>
-        <v>1.72266429913721E-017</v>
+        <v>0</v>
       </c>
       <c r="F33" s="41" t="n">
         <f aca="false">F$12*E33+F$13*E32+F$14*E31+F$15*E30+F$16*E29+F$17*E28</f>
-        <v>6.14448978334277E-016</v>
+        <v>0</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>201</v>
@@ -6724,15 +6724,15 @@
       </c>
       <c r="D34" s="41" t="n">
         <f aca="false">D$15*C31+D$16*C30+D$17*C29</f>
-        <v>2.57164906625409E-022</v>
+        <v>0</v>
       </c>
       <c r="E34" s="41" t="n">
         <f aca="false">E$12*D34+E$13*D33+E$14*D32+E$15*D31+E$16*D30+E$17*D29</f>
-        <v>1.63842132168651E-019</v>
+        <v>0</v>
       </c>
       <c r="F34" s="41" t="n">
         <f aca="false">F$12*E34+F$13*E33+F$14*E32+F$15*E31+F$16*E30+F$17*E29</f>
-        <v>9.43969457170647E-018</v>
+        <v>0</v>
       </c>
       <c r="H34" s="6" t="s">
         <v>202</v>
@@ -6754,15 +6754,15 @@
       </c>
       <c r="D35" s="41" t="n">
         <f aca="false">D$16*C31+D$17*C30</f>
-        <v>5.70957658733089E-025</v>
+        <v>0</v>
       </c>
       <c r="E35" s="41" t="n">
         <f aca="false">E$12*D35+E$13*D34+E$14*D33+E$15*D32+E$16*D31+E$17*D30</f>
-        <v>1.2661089061011E-021</v>
+        <v>0</v>
       </c>
       <c r="F35" s="41" t="n">
         <f aca="false">F$12*E35+F$13*E34+F$14*E33+F$15*E32+F$16*E31+F$17*E30</f>
-        <v>1.24302211348752E-019</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6777,15 +6777,15 @@
       </c>
       <c r="D36" s="41" t="n">
         <f aca="false">D$17*C31</f>
-        <v>5.91563797685812E-028</v>
+        <v>0</v>
       </c>
       <c r="E36" s="41" t="n">
         <f aca="false">E$12*D36+E$13*D35+E$14*D34+E$15*D33+E$16*D32+E$17*D31</f>
-        <v>7.82715055058459E-024</v>
+        <v>0</v>
       </c>
       <c r="F36" s="41" t="n">
         <f aca="false">F$12*E36+F$13*E35+F$14*E34+F$15*E33+F$16*E32+F$17*E31</f>
-        <v>1.40037247695474E-021</v>
+        <v>0</v>
       </c>
       <c r="H36" s="4" t="s">
         <v>203</v>
@@ -6806,11 +6806,11 @@
       </c>
       <c r="E37" s="41" t="n">
         <f aca="false">E$13*D36+E$14*D35+E$15*D34+E$16*D33+E$17*D32</f>
-        <v>3.78027595275189E-026</v>
+        <v>0</v>
       </c>
       <c r="F37" s="41" t="n">
         <f aca="false">F$12*E37+F$13*E36+F$14*E35+F$15*E34+F$16*E33+F$17*E32</f>
-        <v>1.34456700930746E-023</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6828,11 +6828,11 @@
       </c>
       <c r="E38" s="41" t="n">
         <f aca="false">E$14*D36+E$15*D35+E$16*D34+E$17*D33</f>
-        <v>1.37467973086559E-028</v>
+        <v>0</v>
       </c>
       <c r="F38" s="41" t="n">
         <f aca="false">F$12*E38+F$13*E37+F$14*E36+F$15*E35+F$16*E34+F$17*E33</f>
-        <v>1.09352945603514E-025</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6850,11 +6850,11 @@
       </c>
       <c r="E39" s="41" t="n">
         <f aca="false">E$15*D36+E$16*D35+E$17*D34</f>
-        <v>3.54090596874055E-031</v>
+        <v>0</v>
       </c>
       <c r="F39" s="41" t="n">
         <f aca="false">F$12*E39+F$13*E38+F$14*E37+F$15*E36+F$16*E35+F$17*E34</f>
-        <v>7.46617202858622E-028</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6872,11 +6872,11 @@
       </c>
       <c r="E40" s="41" t="n">
         <f aca="false">E$16*D36+E$17*D35</f>
-        <v>5.7603923070847E-034</v>
+        <v>0</v>
       </c>
       <c r="F40" s="41" t="n">
         <f aca="false">F$12*E40+F$13*E39+F$14*E38+F$15*E37+F$16*E36+F$17*E35</f>
-        <v>4.22559657077549E-030</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6894,11 +6894,11 @@
       </c>
       <c r="E41" s="41" t="n">
         <f aca="false">E$17*D36</f>
-        <v>4.45123471827615E-037</v>
+        <v>0</v>
       </c>
       <c r="F41" s="41" t="n">
         <f aca="false">F$12*E41+F$13*E40+F$14*E39+F$15*E38+F$16*E37+F$17*E36</f>
-        <v>1.94737889853518E-032</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6919,7 +6919,7 @@
       </c>
       <c r="F42" s="41" t="n">
         <f aca="false">F$13*E41+F$14*E40+F$15*E39+F$16*E38+F$17*E37</f>
-        <v>7.12258949019275E-035</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6940,7 +6940,7 @@
       </c>
       <c r="F43" s="41" t="n">
         <f aca="false">F$14*E41+F$15*E40+F$16*E39+F$17*E38</f>
-        <v>1.98933324194733E-037</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6961,7 +6961,7 @@
       </c>
       <c r="F44" s="41" t="n">
         <f aca="false">F$15*E41+F$16*E40+F$17*E39</f>
-        <v>3.98592241307424E-040</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="F45" s="41" t="n">
         <f aca="false">F$16*E41+F$17*E40</f>
-        <v>5.1023593580933E-043</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7003,7 +7003,7 @@
       </c>
       <c r="F46" s="41" t="n">
         <f aca="false">F$17*E41</f>
-        <v>3.13509023538759E-046</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>